<commit_message>
docs: Rekonstruktions-MDs 13.05.2026 + Datendateien
</commit_message>
<xml_diff>
--- a/Daten/vorfeldmit/Vorfeldmitarbeiter_2026_05_06.xlsx
+++ b/Daten/vorfeldmit/Vorfeldmitarbeiter_2026_05_06.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vorfeldmitarbeiter" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Vorfeldmitarbeiter'!$A$1:$H$9</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,21 +30,40 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00222222"/>
-      <sz val="13"/>
+      <color rgb="00000000"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="26"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="22"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="11"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -50,31 +71,10 @@
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001565A8"/>
-        <bgColor rgb="001565A8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001B5E20"/>
-        <bgColor rgb="001B5E20"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E65100"/>
-        <bgColor rgb="00E65100"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004527A0"/>
-        <bgColor rgb="004527A0"/>
-      </patternFill>
+      <patternFill patternType="solid"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -83,42 +83,201 @@
       <diagonal/>
     </border>
     <border>
+      <left>
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left>
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="00C8D2DC"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
-        <color rgb="00C8D2DC"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00C8D2DC"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C8D2DC"/>
+        <color rgb="00000000"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -483,119 +642,210 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="52" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DRK KV Köln e.V.  –  Vorfeldmitarbeiter  –  Sanitätsstation CGN        Datum: 06.05.2026</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    DRK KV Köln e.V. </t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Vorfeldmitarbeiter</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr"/>
     </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Gruppe / Zeit</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+    <row r="2" ht="38" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>06.05.2026</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Mitarbeiter 1</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Mitarbeiter 2</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Mitarbeiter 3</t>
         </is>
       </c>
+      <c r="H2" s="4" t="n"/>
     </row>
-    <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="52" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Gruppe 1
 09:00 – 14:00 Uhr</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Gablitschka</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Kurthen</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Spinczyk</t>
-        </is>
-      </c>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Cemal [T10]</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Campolo [T, EM]</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Kalbfleisch [T10]</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="n"/>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4" ht="52" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Gruppe 2
 14:00 – 19:00 Uhr</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Kalbfleisch</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Stoll</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Walke</t>
-        </is>
-      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Kumuini [T]</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Stoll [T10]</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Touahni [T]</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="n"/>
     </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Gruppe 3
 19:00 – 00:00 Uhr</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Singh</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Weigel</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Mohammed</t>
-        </is>
-      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Kleeberg [N, EM]</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Wahlen [N]</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Weigel [N]</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Bearbeitung</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="8" t="inlineStr"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="n"/>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Groß</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>06.05.2026</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+  <mergeCells count="25">
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="C1:F1"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>